<commit_message>
update product center grid view
</commit_message>
<xml_diff>
--- a/src/data/website-data.xlsx
+++ b/src/data/website-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lyanc\VScodeProgram\inteplast_home_page_tw\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65908CA3-C7F8-496D-8FA9-D18DB64E2D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D3BCB4-6025-437A-B672-09836E07E126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="清潔袋" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="238">
   <si>
     <t>產品系列</t>
   </si>
@@ -62,12 +62,15 @@
     <t>10L</t>
   </si>
   <si>
-    <t>40 × 50 cm</t>
+    <t>特小</t>
   </si>
   <si>
     <t>張/捲</t>
   </si>
   <si>
+    <t>透明</t>
+  </si>
+  <si>
     <t>15L</t>
   </si>
   <si>
@@ -161,6 +164,9 @@
     <t>本色 / 紅 / 藍 / 黑 / 綠</t>
   </si>
   <si>
+    <t>拉繩醫療袋</t>
+  </si>
+  <si>
     <t>8L</t>
   </si>
   <si>
@@ -170,6 +176,9 @@
     <t>張</t>
   </si>
   <si>
+    <t>紅</t>
+  </si>
+  <si>
     <t>52 × 55 cm</t>
   </si>
   <si>
@@ -701,15 +710,10 @@
     <t>※ 工作表名稱與欄位標題請勿更改，網站是依名稱找資料的。</t>
   </si>
   <si>
-    <t>大</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>中</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>小</t>
+    <t>41 × 50 cm</t>
+  </si>
+  <si>
+    <t>12L</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -719,125 +723,21 @@
         <rFont val="Microsoft JhengHei"/>
         <family val="2"/>
       </rPr>
-      <t>掌寬</t>
+      <t>超</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Microsoft JhengHei"/>
+        <rFont val="微軟正黑體"/>
         <family val="2"/>
         <charset val="136"/>
       </rPr>
-      <t>食指至小拇指</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>) 8.5~9.5cm</t>
+      <t>小</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Microsoft JhengHei"/>
-        <family val="2"/>
-      </rPr>
-      <t>掌寬</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Microsoft JhengHei"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t>食指至小拇指</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Microsoft JhengHei"/>
-        <family val="2"/>
-      </rPr>
-      <t>小於</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>7.5cm</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Microsoft JhengHei"/>
-        <family val="2"/>
-      </rPr>
-      <t>掌寬</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Microsoft JhengHei"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t>食指至小拇指</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>) 7.5~8.5cm</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>超小</t>
+    <t>38 × 45 cm</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -854,16 +754,8 @@
       <rPr>
         <sz val="11"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
+      <t xml:space="preserve"> / </t>
     </r>
     <r>
       <rPr>
@@ -877,6 +769,18 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>中</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>大</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>小</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -884,16 +788,19 @@
         <family val="2"/>
         <charset val="136"/>
       </rPr>
-      <t>拉繩</t>
+      <t>中</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <rFont val="Microsoft JhengHei"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>感染</t>
+      <t xml:space="preserve"> </t>
     </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -901,19 +808,7 @@
         <family val="2"/>
         <charset val="136"/>
       </rPr>
-      <t>袋</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="細明體"/>
-        <family val="3"/>
-        <charset val="136"/>
-      </rPr>
-      <t>粉色</t>
+      <t>大</t>
     </r>
     <r>
       <rPr>
@@ -921,27 +816,27 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> / </t>
+      <t xml:space="preserve"> </t>
     </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7.5cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>9.5cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
-        <rFont val="細明體"/>
-        <family val="3"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
         <charset val="136"/>
       </rPr>
-      <t>藍色</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Microsoft JhengHei"/>
-        <family val="2"/>
-      </rPr>
-      <t>透明</t>
+      <t>10</t>
     </r>
     <r>
       <rPr>
@@ -949,54 +844,8 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> / </t>
+      <t>cm</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微軟正黑體"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t>黑色</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微軟正黑體"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t>紅</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Microsoft JhengHei"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t>色</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>12L</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>特小</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>38 × 45 cm</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>透明</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1004,7 +853,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1023,18 +872,12 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="微軟正黑體"/>
-      <family val="2"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <name val="微軟正黑體"/>
       <family val="2"/>
       <charset val="136"/>
     </font>
@@ -1051,14 +894,8 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="細明體"/>
-      <family val="3"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="3"/>
+      <family val="2"/>
       <charset val="136"/>
     </font>
   </fonts>
@@ -1090,24 +927,18 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1447,11 +1278,7 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1484,11 +1311,11 @@
       <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>228</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>236</v>
       </c>
       <c r="E2">
         <v>100</v>
@@ -1496,7 +1323,7 @@
       <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>229</v>
       </c>
     </row>
@@ -1504,23 +1331,23 @@
       <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>235</v>
+      <c r="B3" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>225</v>
       </c>
       <c r="E3">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>237</v>
+      <c r="G3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1528,13 +1355,13 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4">
         <v>72</v>
@@ -1543,7 +1370,7 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1551,13 +1378,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5">
         <v>54</v>
@@ -1566,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1574,13 +1401,13 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E6">
         <v>30</v>
@@ -1589,7 +1416,7 @@
         <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1597,13 +1424,13 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7">
         <v>22</v>
@@ -1612,7 +1439,7 @@
         <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1620,13 +1447,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E8">
         <v>16</v>
@@ -1635,7 +1462,7 @@
         <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1643,13 +1470,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E9">
         <v>28</v>
@@ -1658,7 +1485,7 @@
         <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1666,13 +1493,13 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E10">
         <v>10</v>
@@ -1681,7 +1508,7 @@
         <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1689,13 +1516,13 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E11">
         <v>27</v>
@@ -1704,181 +1531,181 @@
         <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+      <c r="G17" t="s">
         <v>25</v>
-      </c>
-      <c r="C17" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G17" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D18" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C20" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C22" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C23" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G23" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1891,15 +1718,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
@@ -1925,300 +1743,282 @@
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="2" t="s">
-        <v>230</v>
+      <c r="A2" t="s">
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E2">
         <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>233</v>
+        <v>46</v>
+      </c>
+      <c r="G2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="2" t="s">
-        <v>230</v>
+      <c r="A3" t="s">
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E3">
         <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>233</v>
+        <v>46</v>
+      </c>
+      <c r="G3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="2" t="s">
-        <v>230</v>
+      <c r="A4" t="s">
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E4">
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>233</v>
+        <v>46</v>
+      </c>
+      <c r="G4" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="2" t="s">
-        <v>230</v>
+      <c r="A5" t="s">
+        <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E5">
         <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>233</v>
+        <v>46</v>
+      </c>
+      <c r="G5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="2" t="s">
-        <v>230</v>
+      <c r="A6" t="s">
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E6">
         <v>12</v>
       </c>
       <c r="F6" t="s">
-        <v>44</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>233</v>
+        <v>46</v>
+      </c>
+      <c r="G6" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7">
         <v>24</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>232</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E8">
         <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>232</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E9">
         <v>14</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="15">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E10">
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>231</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E11">
         <v>15</v>
       </c>
       <c r="F11" t="s">
-        <v>51</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>232</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E12">
         <v>20</v>
       </c>
       <c r="F12" t="s">
-        <v>53</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>232</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G13" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G14" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G15" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G16" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -2232,7 +2032,9 @@
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2261,274 +2063,274 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E2">
         <v>360</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E3">
         <v>255</v>
       </c>
       <c r="F3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E4">
         <v>183</v>
       </c>
       <c r="F4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E5">
         <v>146</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E6">
         <v>99</v>
       </c>
       <c r="F6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E7">
         <v>79</v>
       </c>
       <c r="F7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D8" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E8">
         <v>52</v>
       </c>
       <c r="F8" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D9" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E9">
         <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D10" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E10">
         <v>22</v>
       </c>
       <c r="F10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E11">
         <v>1822</v>
       </c>
       <c r="F11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D12" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E12">
         <v>1275</v>
       </c>
       <c r="F12" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E13">
         <v>897</v>
       </c>
       <c r="F13" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E14">
         <v>708</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D15" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E15">
         <v>472</v>
       </c>
       <c r="F15" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D16" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E16">
         <v>367</v>
       </c>
       <c r="F16" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B17" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D17" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E17">
         <v>236</v>
       </c>
       <c r="F17" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2542,9 +2344,10 @@
   <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2572,347 +2375,347 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E2">
         <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E3">
         <v>100</v>
       </c>
       <c r="F3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E4">
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E5">
         <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D6" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E6">
         <v>100</v>
       </c>
       <c r="F6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D7" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E7">
         <v>100</v>
       </c>
       <c r="F7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D8" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E8">
         <v>100</v>
       </c>
       <c r="F8" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B9" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D9" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E9">
         <v>100</v>
       </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D10" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E10">
         <v>100</v>
       </c>
       <c r="F10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E11">
         <v>100</v>
       </c>
       <c r="F11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B12" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D12" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E12">
         <v>100</v>
       </c>
       <c r="F12" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D13" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E13">
         <v>100</v>
       </c>
       <c r="F13" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D14" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E14">
         <v>100</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D15" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E15">
         <v>100</v>
       </c>
       <c r="F15" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>111</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>223</v>
+        <v>114</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>230</v>
       </c>
       <c r="E16">
         <v>45</v>
       </c>
       <c r="F16" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>111</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>222</v>
+        <v>114</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>231</v>
       </c>
       <c r="E17">
         <v>48</v>
       </c>
       <c r="F17" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>113</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>224</v>
+        <v>116</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>232</v>
       </c>
       <c r="D18" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E18">
         <v>40</v>
       </c>
       <c r="F18" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>113</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>223</v>
+        <v>116</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>230</v>
       </c>
       <c r="D19" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E19">
         <v>30</v>
       </c>
       <c r="F19" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>113</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>222</v>
+        <v>116</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>231</v>
       </c>
       <c r="D20" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E20">
         <v>16</v>
       </c>
       <c r="F20" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="E21">
         <v>45</v>
       </c>
       <c r="F21" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="E22">
         <v>48</v>
       </c>
       <c r="F22" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2926,9 +2729,11 @@
   <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2956,83 +2761,83 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>226</v>
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>227</v>
+        <v>17</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>225</v>
+        <v>20</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -3079,165 +2884,157 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="147.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.88671875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="G2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="G3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B4" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C4" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="G4" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="G5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F6" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C7" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="G7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -3250,137 +3047,133 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="142.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.6640625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B6" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B9" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B10" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B11" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B12" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B13" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B15" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B16" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -3396,137 +3189,137 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edit product list excel
</commit_message>
<xml_diff>
--- a/src/data/website-data.xlsx
+++ b/src/data/website-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lyanc\VScodeProgram\inteplast_home_page_tw\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C7F4A06-BD8E-4B94-A92B-FC44D01412FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B56290-F0AA-4AA7-BEBC-910409A233A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="清潔袋" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="303">
   <si>
     <t>產品系列</t>
   </si>
@@ -62,18 +62,12 @@
     <t>系列代表圖</t>
   </si>
   <si>
-    <t>連捲清潔袋</t>
-  </si>
-  <si>
     <t>10L</t>
   </si>
   <si>
     <t>特小</t>
   </si>
   <si>
-    <t>40 × 50 cm</t>
-  </si>
-  <si>
     <t>張/捲</t>
   </si>
   <si>
@@ -188,15 +182,9 @@
     <t>透明 / 黑色 / 粉紅 / 藍色</t>
   </si>
   <si>
-    <t>環保清潔袋</t>
-  </si>
-  <si>
     <t>本色 / 紅 / 藍 / 黑 / 綠</t>
   </si>
   <si>
-    <t>拉繩醫療袋</t>
-  </si>
-  <si>
     <t>8L</t>
   </si>
   <si>
@@ -212,9 +200,6 @@
     <t>拉繩感染袋 小.webp</t>
   </si>
   <si>
-    <t>封面-拉繩感染袋.png</t>
-  </si>
-  <si>
     <t>52 × 55 cm</t>
   </si>
   <si>
@@ -290,9 +275,6 @@
     <t>本色 / 黑色</t>
   </si>
   <si>
-    <t>平裝耐熱袋</t>
-  </si>
-  <si>
     <t>四兩</t>
   </si>
   <si>
@@ -443,12 +425,6 @@
     <t>34 × 45 cm</t>
   </si>
   <si>
-    <t>密實袋</t>
-  </si>
-  <si>
-    <t>箱/板</t>
-  </si>
-  <si>
     <t>立體密實袋</t>
   </si>
   <si>
@@ -461,9 +437,6 @@
     <t>26 × 25.5 cm</t>
   </si>
   <si>
-    <t>冷凍袋</t>
-  </si>
-  <si>
     <t>台塑遮蔽防塵膠帶</t>
   </si>
   <si>
@@ -488,22 +461,13 @@
     <t>手套</t>
   </si>
   <si>
-    <t>7.5cm</t>
-  </si>
-  <si>
     <t>手套 小.webp</t>
   </si>
   <si>
     <t>封面-手套.webp</t>
   </si>
   <si>
-    <t>9.5cm</t>
-  </si>
-  <si>
     <t>手套 中.webp</t>
-  </si>
-  <si>
-    <t>10cm</t>
   </si>
   <si>
     <t>手套 大.webp</t>
@@ -849,13 +813,739 @@
   <si>
     <t>其他類</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>41 × 50 cm</t>
+  </si>
+  <si>
+    <t>12L</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>38 × 45 cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>透明</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>黑色</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>超小</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>連捲清潔袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+      </rPr>
+      <t>特</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>小</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>連捲清潔袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+      </rPr>
+      <t>特</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>大</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>環保清潔袋.webp</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>拉繩感染袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.png</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>蔬果袋</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>耐熱袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <t>保鮮耐熱袋</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>20 × 30 cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>28 × 41 cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>保鮮耐熱袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>保鮮耐熱袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>小</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>保鮮耐熱袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>大</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <t>張</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>平裝耐熱袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>營潔平裝耐熱袋</t>
+  </si>
+  <si>
+    <t>台塑清潔袋</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>台塑環保清潔袋</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>台塑拉繩感染清潔袋</t>
+  </si>
+  <si>
+    <t>台塑拉繩清潔袋</t>
+  </si>
+  <si>
+    <r>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>台塑拉繩清潔袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>夾鏈袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>立體密食袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>小</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>立體密食袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>中</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>立體密食袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>大</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+      </rPr>
+      <t>張</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>盒</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>台塑保鮮密實袋</t>
+  </si>
+  <si>
+    <t>台塑夾鏈袋</t>
+  </si>
+  <si>
+    <t>17.8 × 19.5 cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>密食袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>中</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <t>26.8 × 27.3 cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>密食袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>大</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>冷凍袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>大</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <t>冷凍袋 中.webp</t>
+  </si>
+  <si>
+    <t>台塑保鮮冷凍袋</t>
+  </si>
+  <si>
+    <t>台塑立體密實袋</t>
+  </si>
+  <si>
+    <r>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>台塑夾鏈袋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.webp</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>台塑遮蔽防塵膠帶</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.png</t>
+    </r>
+  </si>
+  <si>
+    <t>7.5 cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>8.5~9.5 cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7.5~8.5 cm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>封面</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>-Scale Sheet.jpg</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -882,6 +1572,47 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Microsoft JhengHei"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Microsoft JhengHei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="2"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="細明體"/>
+      <family val="2"/>
+      <charset val="136"/>
     </font>
   </fonts>
   <fills count="3">
@@ -912,7 +1643,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -921,6 +1652,21 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1257,8 +2003,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
   <cols>
     <col min="1" max="1" width="17.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.77734375" bestFit="1" customWidth="1"/>
@@ -1268,10 +2014,10 @@
     <col min="6" max="6" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="26" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="14.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1300,412 +2046,444 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="14.4">
       <c r="A2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
+      <c r="C2" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>259</v>
       </c>
       <c r="E2">
         <v>100</v>
       </c>
       <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="H2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:9" ht="14.4">
+      <c r="A3" t="s">
+        <v>277</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="14.4">
+      <c r="A4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="I2" t="s">
+      <c r="C4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="D4" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E4">
+        <v>72</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
+      <c r="H4" t="s">
         <v>19</v>
       </c>
-      <c r="E3">
-        <v>72</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" t="s">
+    </row>
+    <row r="5" spans="1:9" ht="14.4">
+      <c r="A5" t="s">
+        <v>277</v>
+      </c>
+      <c r="B5" t="s">
         <v>20</v>
       </c>
-      <c r="H3" t="s">
+      <c r="C5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="D5" t="s">
         <v>22</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E5">
+        <v>54</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" t="s">
         <v>23</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="6" spans="1:9" ht="14.4">
+      <c r="A6" t="s">
+        <v>277</v>
+      </c>
+      <c r="B6" t="s">
         <v>24</v>
       </c>
-      <c r="E4">
-        <v>54</v>
-      </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="C6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="D6" t="s">
         <v>26</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E6">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" t="s">
         <v>27</v>
       </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="7" spans="1:9" ht="14.4">
+      <c r="A7" t="s">
+        <v>277</v>
+      </c>
+      <c r="B7" t="s">
         <v>28</v>
       </c>
-      <c r="E5">
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s">
         <v>30</v>
       </c>
-      <c r="F5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="E7">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
         <v>31</v>
       </c>
-      <c r="D6" t="s">
+      <c r="H7" s="4" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="14.4">
+      <c r="A8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B8" t="s">
         <v>32</v>
       </c>
-      <c r="E6">
-        <v>22</v>
-      </c>
-      <c r="F6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="C8" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="D8" t="s">
         <v>34</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E8">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" t="s">
         <v>35</v>
       </c>
-      <c r="D7" t="s">
+    </row>
+    <row r="9" spans="1:9" ht="14.4">
+      <c r="A9" t="s">
+        <v>277</v>
+      </c>
+      <c r="B9" t="s">
         <v>36</v>
       </c>
-      <c r="E7">
-        <v>16</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="C9" t="s">
         <v>33</v>
       </c>
-      <c r="H7" t="s">
+      <c r="D9" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="E9">
+        <v>28</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" t="s">
         <v>35</v>
       </c>
-      <c r="D8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8">
-        <v>28</v>
-      </c>
-      <c r="F8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" t="s">
-        <v>33</v>
-      </c>
-      <c r="H8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" t="s">
-        <v>42</v>
-      </c>
-      <c r="E9">
-        <v>10</v>
-      </c>
-      <c r="F9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" t="s">
-        <v>33</v>
-      </c>
-      <c r="H9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:9" ht="14.4">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>277</v>
       </c>
       <c r="B10" t="s">
         <v>38</v>
       </c>
       <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="14.4">
+      <c r="A11" t="s">
+        <v>277</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11">
+        <v>27</v>
+      </c>
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="14.4">
+      <c r="A12" t="s">
         <v>44</v>
       </c>
-      <c r="D10" t="s">
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
         <v>45</v>
       </c>
-      <c r="E10">
-        <v>27</v>
-      </c>
-      <c r="F10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="D12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="14.4">
+      <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="14.4">
+      <c r="A14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="14.4">
+      <c r="A15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="14.4">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="14.4">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" t="s">
         <v>33</v>
       </c>
-      <c r="H10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" t="s">
-        <v>48</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="D17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="14.4">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15">
+      <c r="A19" t="s">
+        <v>278</v>
+      </c>
+      <c r="C19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19" t="s">
+        <v>49</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="14.4">
+      <c r="A20" t="s">
+        <v>278</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="14.4">
+      <c r="A21" t="s">
+        <v>278</v>
+      </c>
+      <c r="C21" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="14.4">
+      <c r="A22" t="s">
+        <v>278</v>
+      </c>
+      <c r="C22" t="s">
+        <v>29</v>
+      </c>
+      <c r="G22" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="14.4">
+      <c r="A23" t="s">
+        <v>278</v>
+      </c>
+      <c r="C23" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="G23" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D13" t="s">
-        <v>24</v>
-      </c>
-      <c r="G13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" t="s">
-        <v>28</v>
-      </c>
-      <c r="G14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" t="s">
-        <v>32</v>
-      </c>
-      <c r="G15" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" t="s">
-        <v>36</v>
-      </c>
-      <c r="G16" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" t="s">
-        <v>42</v>
-      </c>
-      <c r="G17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" t="s">
-        <v>27</v>
-      </c>
-      <c r="G18" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>51</v>
-      </c>
-      <c r="C19" t="s">
-        <v>18</v>
-      </c>
-      <c r="G19" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" t="s">
-        <v>23</v>
-      </c>
-      <c r="G20" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" t="s">
-        <v>31</v>
-      </c>
-      <c r="G21" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" t="s">
-        <v>35</v>
-      </c>
-      <c r="G22" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1717,18 +2495,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
   <cols>
-    <col min="1" max="1" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.77734375" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="14.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1757,319 +2536,322 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>53</v>
+    <row r="2" spans="1:9" ht="15">
+      <c r="A2" s="6" t="s">
+        <v>279</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E2">
         <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
-      </c>
-      <c r="I2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="15">
+      <c r="A3" s="6" t="s">
+        <v>279</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E3">
         <v>22</v>
       </c>
       <c r="F3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" t="s">
         <v>56</v>
       </c>
-      <c r="G3" t="s">
+    </row>
+    <row r="4" spans="1:9" ht="15">
+      <c r="A4" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="B4" t="s">
         <v>57</v>
       </c>
-      <c r="H3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" t="s">
-        <v>62</v>
-      </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E4">
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>53</v>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="15">
+      <c r="A5" s="6" t="s">
+        <v>279</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E5">
         <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>53</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="15">
+      <c r="A6" s="6" t="s">
+        <v>279</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E6">
         <v>12</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="14.4">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>280</v>
       </c>
       <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
         <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>28</v>
       </c>
       <c r="E7">
         <v>24</v>
       </c>
       <c r="F7" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H7" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="14.4">
       <c r="A8" t="s">
-        <v>69</v>
+        <v>280</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E8">
         <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="14.4">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>280</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E9">
         <v>14</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="14.4">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>280</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E10">
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="14.4">
       <c r="A11" t="s">
-        <v>69</v>
+        <v>280</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E11">
         <v>15</v>
       </c>
       <c r="F11" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="14.4">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>280</v>
       </c>
       <c r="B12" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D12" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E12">
         <v>20</v>
       </c>
       <c r="F12" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H12" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="14.4">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G13" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="14.4">
       <c r="A14" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G14" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="14.4">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="14.4">
       <c r="A16" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G16" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2080,19 +2862,20 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L20"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="14.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2121,276 +2904,339 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="15">
       <c r="A2" t="s">
-        <v>85</v>
+        <v>276</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E2">
         <v>360</v>
       </c>
       <c r="F2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="14.4">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>276</v>
       </c>
       <c r="B3" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D3" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E3">
         <v>255</v>
       </c>
       <c r="F3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="14.4">
       <c r="A4" t="s">
+        <v>276</v>
+      </c>
+      <c r="B4" t="s">
         <v>85</v>
       </c>
-      <c r="B4" t="s">
-        <v>91</v>
-      </c>
       <c r="D4" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E4">
         <v>183</v>
       </c>
       <c r="F4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="14.4">
+      <c r="A5" t="s">
+        <v>276</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B5" t="s">
-        <v>93</v>
-      </c>
-      <c r="D5" t="s">
-        <v>94</v>
       </c>
       <c r="E5">
         <v>146</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="14.4">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>276</v>
       </c>
       <c r="B6" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D6" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E6">
         <v>99</v>
       </c>
       <c r="F6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="14.4">
       <c r="A7" t="s">
-        <v>85</v>
+        <v>276</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D7" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E7">
         <v>79</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="14.4">
       <c r="A8" t="s">
-        <v>85</v>
+        <v>276</v>
       </c>
       <c r="B8" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D8" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E8">
         <v>52</v>
       </c>
       <c r="F8" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="L8" s="8"/>
+    </row>
+    <row r="9" spans="1:12" ht="14.4">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>276</v>
       </c>
       <c r="B9" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D9" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E9">
         <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="L9" s="8"/>
+    </row>
+    <row r="10" spans="1:12" ht="14.4">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>276</v>
       </c>
       <c r="B10" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D10" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="E10">
         <v>22</v>
       </c>
       <c r="F10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="L10" s="8"/>
+    </row>
+    <row r="11" spans="1:12" ht="15">
       <c r="A11" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D11" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E11">
         <v>1822</v>
       </c>
       <c r="F11" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="L11" s="8"/>
+    </row>
+    <row r="12" spans="1:12" ht="14.4">
       <c r="A12" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B12" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D12" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E12">
         <v>1275</v>
       </c>
       <c r="F12" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="L12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" ht="14.4">
       <c r="A13" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D13" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E13">
         <v>897</v>
       </c>
       <c r="F13" t="s">
+        <v>82</v>
+      </c>
+      <c r="L13" s="8"/>
+    </row>
+    <row r="14" spans="1:12" ht="14.4">
+      <c r="A14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>105</v>
-      </c>
-      <c r="B14" t="s">
-        <v>93</v>
-      </c>
-      <c r="D14" t="s">
-        <v>94</v>
       </c>
       <c r="E14">
         <v>708</v>
       </c>
       <c r="F14" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="L14" s="8"/>
+    </row>
+    <row r="15" spans="1:12" ht="14.4">
       <c r="A15" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B15" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D15" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E15">
         <v>472</v>
       </c>
       <c r="F15" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="L15" s="8"/>
+    </row>
+    <row r="16" spans="1:12" ht="14.4">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D16" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E16">
         <v>367</v>
       </c>
       <c r="F16" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="L16" s="8"/>
+    </row>
+    <row r="17" spans="1:9" ht="14.4">
       <c r="A17" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D17" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E17">
         <v>236</v>
       </c>
       <c r="F17" t="s">
-        <v>88</v>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="14.4">
+      <c r="A18" s="7" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15">
+      <c r="A19" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="E19">
+        <v>100</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="15">
+      <c r="A20" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="E20">
+        <v>101</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -2402,18 +3248,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="14.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2442,349 +3289,394 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="14.4">
       <c r="A2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B2" t="s">
-        <v>108</v>
+        <v>288</v>
+      </c>
+      <c r="C2" t="s">
+        <v>102</v>
       </c>
       <c r="D2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="E2">
         <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="14.4">
       <c r="A3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B3" t="s">
-        <v>110</v>
+        <v>101</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
       </c>
       <c r="D3" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E3">
         <v>100</v>
       </c>
       <c r="F3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="14.4">
       <c r="A4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" t="s">
         <v>107</v>
-      </c>
-      <c r="B4" t="s">
-        <v>112</v>
-      </c>
-      <c r="D4" t="s">
-        <v>113</v>
       </c>
       <c r="E4">
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="14.4">
       <c r="A5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B5" t="s">
-        <v>114</v>
+        <v>101</v>
+      </c>
+      <c r="C5" t="s">
+        <v>108</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E5">
         <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="14.4">
       <c r="A6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B6" t="s">
-        <v>116</v>
+        <v>101</v>
+      </c>
+      <c r="C6" t="s">
+        <v>110</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="E6">
         <v>100</v>
       </c>
       <c r="F6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="14.4">
       <c r="A7" t="s">
-        <v>107</v>
-      </c>
-      <c r="B7" t="s">
-        <v>118</v>
+        <v>101</v>
+      </c>
+      <c r="C7" t="s">
+        <v>112</v>
       </c>
       <c r="D7" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E7">
         <v>100</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="14.4">
       <c r="A8" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" t="s">
-        <v>120</v>
+        <v>101</v>
+      </c>
+      <c r="C8" t="s">
+        <v>114</v>
       </c>
       <c r="D8" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="E8">
         <v>100</v>
       </c>
       <c r="F8" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="14.4">
       <c r="A9" t="s">
-        <v>107</v>
-      </c>
-      <c r="B9" t="s">
-        <v>122</v>
+        <v>101</v>
+      </c>
+      <c r="C9" t="s">
+        <v>116</v>
       </c>
       <c r="D9" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="E9">
         <v>100</v>
       </c>
       <c r="F9" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="14.4">
       <c r="A10" t="s">
-        <v>107</v>
-      </c>
-      <c r="B10" t="s">
-        <v>124</v>
+        <v>101</v>
+      </c>
+      <c r="C10" t="s">
+        <v>118</v>
       </c>
       <c r="D10" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E10">
         <v>100</v>
       </c>
       <c r="F10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="14.4">
       <c r="A11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" t="s">
-        <v>126</v>
+        <v>101</v>
+      </c>
+      <c r="C11" t="s">
+        <v>120</v>
       </c>
       <c r="D11" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="E11">
         <v>100</v>
       </c>
       <c r="F11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="14.4">
       <c r="A12" t="s">
-        <v>107</v>
-      </c>
-      <c r="B12" t="s">
-        <v>128</v>
+        <v>101</v>
+      </c>
+      <c r="C12" t="s">
+        <v>122</v>
       </c>
       <c r="D12" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E12">
         <v>100</v>
       </c>
       <c r="F12" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="14.4">
       <c r="A13" t="s">
-        <v>107</v>
-      </c>
-      <c r="B13" t="s">
-        <v>130</v>
+        <v>101</v>
+      </c>
+      <c r="C13" t="s">
+        <v>124</v>
       </c>
       <c r="D13" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E13">
         <v>100</v>
       </c>
       <c r="F13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="14.4">
       <c r="A14" t="s">
-        <v>107</v>
-      </c>
-      <c r="B14" t="s">
-        <v>132</v>
+        <v>101</v>
+      </c>
+      <c r="C14" t="s">
+        <v>126</v>
       </c>
       <c r="D14" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E14">
         <v>100</v>
       </c>
       <c r="F14" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="14.4">
       <c r="A15" t="s">
-        <v>107</v>
-      </c>
-      <c r="B15" t="s">
-        <v>134</v>
+        <v>101</v>
+      </c>
+      <c r="C15" t="s">
+        <v>128</v>
       </c>
       <c r="D15" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E15">
         <v>100</v>
       </c>
       <c r="F15" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15">
       <c r="A16" t="s">
-        <v>136</v>
+        <v>287</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>260</v>
+        <v>248</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>289</v>
       </c>
       <c r="E16">
-        <v>45</v>
-      </c>
-      <c r="F16" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="15">
       <c r="A17" t="s">
-        <v>136</v>
+        <v>287</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>261</v>
+        <v>249</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>291</v>
       </c>
       <c r="E17">
-        <v>48</v>
-      </c>
-      <c r="F17" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15">
       <c r="A18" t="s">
-        <v>138</v>
+        <v>296</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="D18" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="E18">
         <v>40</v>
       </c>
       <c r="F18" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="14.4">
       <c r="A19" t="s">
-        <v>138</v>
+        <v>296</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="D19" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="E19">
         <v>30</v>
       </c>
       <c r="F19" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="14.4">
       <c r="A20" t="s">
-        <v>138</v>
+        <v>296</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="D20" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="E20">
         <v>16</v>
       </c>
       <c r="F20" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="15">
       <c r="A21" t="s">
-        <v>142</v>
+        <v>295</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>260</v>
+        <v>248</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>289</v>
       </c>
       <c r="E21">
-        <v>45</v>
-      </c>
-      <c r="F21" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="15">
       <c r="A22" t="s">
-        <v>142</v>
+        <v>295</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>261</v>
+        <v>249</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>291</v>
       </c>
       <c r="E22">
-        <v>48</v>
-      </c>
-      <c r="F22" t="s">
-        <v>137</v>
+        <v>14</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -2796,16 +3688,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
   <cols>
     <col min="1" max="1" width="19.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.109375" customWidth="1"/>
+    <col min="9" max="9" width="33.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="14.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2834,97 +3727,100 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="14.4">
       <c r="A2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D2" t="s">
+        <v>135</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="14.4">
+      <c r="A3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="14.4">
+      <c r="A4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="14.4">
+      <c r="A5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="14.4">
+      <c r="A6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="14.4">
+      <c r="A7" t="s">
+        <v>134</v>
+      </c>
+      <c r="D7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="14.4">
+      <c r="A8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="H8" t="s">
+        <v>142</v>
+      </c>
+      <c r="I8" t="s">
         <v>143</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="9" spans="1:9" ht="14.4">
+      <c r="A9" t="s">
+        <v>141</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="H9" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>143</v>
-      </c>
-      <c r="D3" t="s">
+    <row r="10" spans="1:9" ht="14.4">
+      <c r="A10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="H10" t="s">
         <v>145</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>143</v>
-      </c>
-      <c r="D4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>143</v>
-      </c>
-      <c r="D5" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D6" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>143</v>
-      </c>
-      <c r="D7" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" t="s">
-        <v>151</v>
-      </c>
-      <c r="H8" t="s">
-        <v>152</v>
-      </c>
-      <c r="I8" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>154</v>
-      </c>
-      <c r="H9" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>150</v>
-      </c>
-      <c r="C10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" t="s">
-        <v>156</v>
-      </c>
-      <c r="H10" t="s">
-        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -2935,10 +3831,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="14.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2965,6 +3861,11 @@
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="I2" s="6" t="s">
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -2976,7 +3877,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -2987,177 +3888,177 @@
     <col min="7" max="7" width="38.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="14.4">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="14.4">
+      <c r="A2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="14.4">
+      <c r="A3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G3" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="H3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="14.4">
+      <c r="A4" t="s">
         <v>165</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C4" t="s">
         <v>166</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D4" t="s">
         <v>167</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E4" t="s">
         <v>168</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F4" t="s">
         <v>169</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G4" t="s">
         <v>170</v>
       </c>
-      <c r="H2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="H4" t="s">
         <v>171</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="14.4">
+      <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C5" t="s">
         <v>172</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D5" t="s">
         <v>173</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E5" t="s">
         <v>174</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F5" t="s">
         <v>175</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G5" t="s">
         <v>176</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H5" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="6" spans="1:8" ht="14.4">
+      <c r="A6" t="s">
         <v>177</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B6" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="C6" t="s">
         <v>178</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D6" t="s">
         <v>179</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E6" t="s">
         <v>180</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F6" t="s">
         <v>181</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G6" t="s">
         <v>182</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H6" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="14.4">
+      <c r="A7" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C5" t="s">
-        <v>184</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="B7" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C7" t="s">
+        <v>183</v>
+      </c>
+      <c r="G7" t="s">
         <v>185</v>
       </c>
-      <c r="E5" t="s">
-        <v>186</v>
-      </c>
-      <c r="F5" t="s">
-        <v>187</v>
-      </c>
-      <c r="G5" t="s">
-        <v>188</v>
-      </c>
-      <c r="H5" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>189</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="C6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D6" t="s">
-        <v>191</v>
-      </c>
-      <c r="E6" t="s">
-        <v>192</v>
-      </c>
-      <c r="F6" t="s">
-        <v>193</v>
-      </c>
-      <c r="G6" t="s">
-        <v>194</v>
-      </c>
-      <c r="H6" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>195</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="C7" t="s">
-        <v>195</v>
-      </c>
-      <c r="G7" t="s">
-        <v>197</v>
-      </c>
       <c r="H7" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -3169,134 +4070,134 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="14.4">
       <c r="A1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="14.4">
+      <c r="A2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="14.4">
+      <c r="A3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="14.4">
+      <c r="A4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="14.4">
+      <c r="A5" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="14.4">
+      <c r="A6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="14.4">
+      <c r="A7" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="14.4">
+      <c r="A8" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B8" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="9" spans="1:2" ht="14.4">
+      <c r="A9" t="s">
         <v>200</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="14.4">
+      <c r="A10" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B10" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="14.4">
+      <c r="A11" t="s">
         <v>202</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="14.4">
+      <c r="A12" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B12" t="s">
         <v>204</v>
       </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    </row>
+    <row r="13" spans="1:2" ht="14.4">
+      <c r="A13" t="s">
         <v>205</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B13" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="14.4">
+      <c r="A14" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B14" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="14.4">
+      <c r="A15" t="s">
         <v>207</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B15" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="16" spans="1:2" ht="14.4">
+      <c r="A16" t="s">
         <v>209</v>
       </c>
-      <c r="B7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B16" t="s">
         <v>210</v>
-      </c>
-      <c r="B8" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>212</v>
-      </c>
-      <c r="B9" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>213</v>
-      </c>
-      <c r="B10" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>214</v>
-      </c>
-      <c r="B11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>215</v>
-      </c>
-      <c r="B12" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>217</v>
-      </c>
-      <c r="B13" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>218</v>
-      </c>
-      <c r="B14" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>219</v>
-      </c>
-      <c r="B15" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>221</v>
-      </c>
-      <c r="B16" t="s">
-        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -3308,203 +4209,203 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:A45"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="14.4">
       <c r="A1" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="14.4"/>
+    <row r="3" spans="1:1" ht="14.4">
+      <c r="A3" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="14.4"/>
+    <row r="5" spans="1:1" ht="14.4">
+      <c r="A5" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="14.4">
+      <c r="A6" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="14.4">
+      <c r="A7" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="14.4">
+      <c r="A8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="14.4">
+      <c r="A9" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="14.4">
+      <c r="A10" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="14.4">
+      <c r="A11" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="14.4">
+      <c r="A12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="14.4">
+      <c r="A13" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="14.4">
+      <c r="A14" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="14.4">
+      <c r="A15" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="16" spans="1:1" ht="14.4">
+      <c r="A16" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="17" spans="1:1" ht="14.4">
+      <c r="A17" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="18" spans="1:1" ht="14.4"/>
+    <row r="19" spans="1:1" ht="14.4">
+      <c r="A19" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="20" spans="1:1" ht="14.4">
+      <c r="A20" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="21" spans="1:1" ht="14.4">
+      <c r="A21" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="22" spans="1:1" ht="14.4">
+      <c r="A22" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="23" spans="1:1" ht="14.4">
+      <c r="A23" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row r="24" spans="1:1" ht="14.4">
+      <c r="A24" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row r="25" spans="1:1" ht="14.4">
+      <c r="A25" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="14.4">
+      <c r="A26" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row r="27" spans="1:1" ht="14.4">
+      <c r="A27" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+    <row r="28" spans="1:1" ht="14.4">
+      <c r="A28" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row r="29" spans="1:1" ht="14.4">
+      <c r="A29" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row r="30" spans="1:1" ht="14.4">
+      <c r="A30" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+    <row r="31" spans="1:1" ht="14.4">
+      <c r="A31" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+    <row r="32" spans="1:1" ht="14.4"/>
+    <row r="33" spans="1:1" ht="14.4">
+      <c r="A33" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+    <row r="34" spans="1:1" ht="14.4">
+      <c r="A34" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+    <row r="35" spans="1:1" ht="14.4">
+      <c r="A35" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+    <row r="36" spans="1:1" ht="14.4"/>
+    <row r="37" spans="1:1" ht="14.4">
+      <c r="A37" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+    <row r="38" spans="1:1" ht="14.4">
+      <c r="A38" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+    <row r="39" spans="1:1" ht="14.4">
+      <c r="A39" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+    <row r="40" spans="1:1" ht="14.4"/>
+    <row r="41" spans="1:1" ht="14.4">
+      <c r="A41" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+    <row r="42" spans="1:1" ht="14.4">
+      <c r="A42" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+    <row r="43" spans="1:1" ht="14.4">
+      <c r="A43" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+    <row r="44" spans="1:1" ht="14.4"/>
+    <row r="45" spans="1:1" ht="14.4">
+      <c r="A45" t="s">
         <v>247</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="33" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="45" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>